<commit_message>
chore: add tracking fields to sample bulk excel
</commit_message>
<xml_diff>
--- a/sample-bulk-import-test.xlsx
+++ b/sample-bulk-import-test.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="49">
   <si>
     <t>Branch Name</t>
   </si>
@@ -34,6 +34,12 @@
     <t>Unit Price</t>
   </si>
   <si>
+    <t>Item Code</t>
+  </si>
+  <si>
+    <t>Serial Number</t>
+  </si>
+  <si>
     <t>Alagar Kovil Registered Office</t>
   </si>
   <si>
@@ -46,9 +52,21 @@
     <t>Boxes</t>
   </si>
   <si>
+    <t>FA-001</t>
+  </si>
+  <si>
+    <t>SN-FA-1001</t>
+  </si>
+  <si>
     <t>Aruldoss Puram Rehabilitation Center</t>
   </si>
   <si>
+    <t>FA-002</t>
+  </si>
+  <si>
+    <t>SN-FA-1002</t>
+  </si>
+  <si>
     <t>KK Nagar Head Office</t>
   </si>
   <si>
@@ -61,9 +79,21 @@
     <t>Packs</t>
   </si>
   <si>
+    <t>A4-500</t>
+  </si>
+  <si>
+    <t>SN-PAPER-01</t>
+  </si>
+  <si>
     <t>Blue Ink Pens</t>
   </si>
   <si>
+    <t>PEN-B-01</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>Lake Area Training Institute (MSCIMHR)</t>
   </si>
   <si>
@@ -73,6 +103,9 @@
     <t>School &amp; Education</t>
   </si>
   <si>
+    <t>MRK-W-01</t>
+  </si>
+  <si>
     <t>Training Manuals</t>
   </si>
   <si>
@@ -82,6 +115,9 @@
     <t>Units</t>
   </si>
   <si>
+    <t>MNL-TR-01</t>
+  </si>
+  <si>
     <t>Alagarkoil Administrative Office</t>
   </si>
   <si>
@@ -91,16 +127,37 @@
     <t>Bottles</t>
   </si>
   <si>
+    <t>HS-500ML</t>
+  </si>
+  <si>
+    <t>SN-HS-500</t>
+  </si>
+  <si>
     <t>Disinfectant Wipes</t>
   </si>
   <si>
+    <t>DW-01</t>
+  </si>
+  <si>
+    <t>SN-DW-123</t>
+  </si>
+  <si>
     <t>Stapler Pins</t>
   </si>
   <si>
+    <t>STP-01</t>
+  </si>
+  <si>
     <t>Chennai Branch</t>
   </si>
   <si>
     <t>Invalid Test Item</t>
+  </si>
+  <si>
+    <t>INV-01</t>
+  </si>
+  <si>
+    <t>SN-INV</t>
   </si>
 </sst>
 </file>
@@ -477,16 +534,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -508,19 +567,25 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <v>45</v>
@@ -531,19 +596,25 @@
       <c r="G2">
         <v>50</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E3">
         <v>30</v>
@@ -554,19 +625,25 @@
       <c r="G3">
         <v>45</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E4">
         <v>150</v>
@@ -577,19 +654,25 @@
       <c r="G4">
         <v>120</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
       </c>
       <c r="E5">
         <v>20</v>
@@ -600,19 +683,25 @@
       <c r="G5">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -623,19 +712,25 @@
       <c r="G6">
         <v>45</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E7">
         <v>200</v>
@@ -646,19 +741,25 @@
       <c r="G7">
         <v>200</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E8">
         <v>25</v>
@@ -669,19 +770,25 @@
       <c r="G8">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E9">
         <v>5</v>
@@ -692,19 +799,25 @@
       <c r="G9">
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>41</v>
+      </c>
+      <c r="I9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E10">
         <v>50</v>
@@ -715,19 +828,25 @@
       <c r="G10">
         <v>45</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -737,6 +856,12 @@
       </c>
       <c r="G11">
         <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>47</v>
+      </c>
+      <c r="I11" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>